<commit_message>
Remove the follow-up form from the result page
Clears lead_endpoint in the content workbook, which hides the form, and
updates the privacy note to match.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011LV79Kwk1BJCCXE63YdDTi
</commit_message>
<xml_diff>
--- a/content/aptara-survey-content.xlsx
+++ b/content/aptara-survey-content.xlsx
@@ -760,7 +760,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Your answers are used only to generate your result. We don't ask for contact details unless you choose to share them.</t>
+          <t>Your answers stay in your browser and are used only to generate your result.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -846,11 +846,7 @@
           <t>lead_endpoint</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>https://formsubmit.co/ajax/karthikeyan@aptaracorp.com</t>
-        </is>
-      </c>
+      <c r="B15" s="5" t="n"/>
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Where follow-up requests are sent. Leave empty to hide the follow-up form.</t>

</xml_diff>

<commit_message>
Remove the follow-up form from the result page (#7)
Clears lead_endpoint in the content workbook, which hides the form, and
updates the privacy note to match.


Claude-Session: https://claude.ai/code/session_011LV79Kwk1BJCCXE63YdDTi

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/aptara-survey-content.xlsx
+++ b/content/aptara-survey-content.xlsx
@@ -760,7 +760,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Your answers are used only to generate your result. We don't ask for contact details unless you choose to share them.</t>
+          <t>Your answers stay in your browser and are used only to generate your result.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -846,11 +846,7 @@
           <t>lead_endpoint</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>https://formsubmit.co/ajax/karthikeyan@aptaracorp.com</t>
-        </is>
-      </c>
+      <c r="B15" s="5" t="n"/>
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Where follow-up requests are sent. Leave empty to hide the follow-up form.</t>

</xml_diff>

<commit_message>
Bring back the follow-up form
Reverts the removal in #7: lead_endpoint is set to FormSubmit again and the
privacy note mentions optional contact details.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011LV79Kwk1BJCCXE63YdDTi
</commit_message>
<xml_diff>
--- a/content/aptara-survey-content.xlsx
+++ b/content/aptara-survey-content.xlsx
@@ -760,7 +760,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Your answers stay in your browser and are used only to generate your result.</t>
+          <t>Your answers are used only to generate your result. We don't ask for contact details unless you choose to share them.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -846,7 +846,11 @@
           <t>lead_endpoint</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>https://formsubmit.co/ajax/karthikeyan@aptaracorp.com</t>
+        </is>
+      </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Where follow-up requests are sent. Leave empty to hide the follow-up form.</t>

</xml_diff>

<commit_message>
Bring back the follow-up form (#8)
Reverts the removal in #7: lead_endpoint is set to FormSubmit again and the
privacy note mentions optional contact details.


Claude-Session: https://claude.ai/code/session_011LV79Kwk1BJCCXE63YdDTi

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/aptara-survey-content.xlsx
+++ b/content/aptara-survey-content.xlsx
@@ -760,7 +760,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Your answers stay in your browser and are used only to generate your result.</t>
+          <t>Your answers are used only to generate your result. We don't ask for contact details unless you choose to share them.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -846,7 +846,11 @@
           <t>lead_endpoint</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>https://formsubmit.co/ajax/karthikeyan@aptaracorp.com</t>
+        </is>
+      </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Where follow-up requests are sent. Leave empty to hide the follow-up form.</t>

</xml_diff>

<commit_message>
Follow-up polish: confirmed Start over, merged guidance, hero example
- Start over asks first (native modal dialog) whenever answers or a result
  would be lost; an untouched first step resets straight away.
- Team size and sourcing write one paragraph, from a rule per pair.
- Priority cards carry an Action tag; cards sharing one are merged, with a
  natural merge note instead of "listed once" wording.
- Delivery advice states the method mix, then one sentence for the main
  challenge, method-specific where it matters. Add rules now apply only
  the highest-priority match per mode.
- The first screen is decided synchronously from saved state, so a refresh
  no longer flashes the landing page.
- Compact, illustrative example result card in the hero, built from the
  real rules; the lower duplicate preview is removed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011LV79Kwk1BJCCXE63YdDTi
</commit_message>
<xml_diff>
--- a/content/aptara-survey-content.xlsx
+++ b/content/aptara-survey-content.xlsx
@@ -523,7 +523,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Rules: Remove hides a section; Replace, Add before and Add after change its text. See docs/recommendation-mapping.md in the repo.</t>
+          <t>Rules: Remove hides a section; Replace, Add before and Add after change its text. Only the highest-Priority rule of each mode applies to a section. Priority cards with the same Action are shown once. See docs/recommendation-mapping.md in the repo.</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2203,6 +2203,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="60" customHeight="1">
@@ -2248,6 +2249,11 @@
           <t>Writing guidance</t>
         </is>
       </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Merge note</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -2283,6 +2289,7 @@
           <t>Names the first priority, using the same words as its heading.</t>
         </is>
       </c>
+      <c r="H3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -2318,6 +2325,7 @@
           <t>Restates the stage they chose, in their terms. Directional, not a diagnosis.</t>
         </is>
       </c>
+      <c r="H4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2353,6 +2361,7 @@
           <t>Heading = the action. Text = what to do. Why = which answer it comes from.</t>
         </is>
       </c>
+      <c r="H5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2385,7 +2394,12 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Heading = the action. Removed by a rule when it repeats the challenge priority.</t>
+          <t>Heading = the action. Merged into an earlier priority when it has the same Action tag.</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>It also supports the business goal you chose for the next 6–12 months.</t>
         </is>
       </c>
     </row>
@@ -2423,6 +2437,11 @@
           <t>The level of process and governance guidance that fits their stage.</t>
         </is>
       </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>It also fits the stage you described ({Q1}).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2455,9 +2474,10 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Single method: advice for that method. MULTI: advice for using several methods together; {Q3} lists them.</t>
-        </is>
-      </c>
+          <t>States the method mix only. A rule adds one sentence chosen by main challenge (and method, where it matters).</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2485,33 +2505,34 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Context card (first sentence)</t>
+          <t>Context card</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Workload advice for their team size. Never assume an internal production team.</t>
-        </is>
-      </c>
+          <t>Replaced by a rule for each team size and sourcing pair, so team and sourcing read as one paragraph. These blocks are the fallback.</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>sourcing</t>
+          <t>next30</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Your team and capacity</t>
+          <t>Next 30 days</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>240</v>
+        <v>260</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
@@ -2520,33 +2541,34 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Context card (second sentence)</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Coordination advice for how work is delivered. Don't prescribe outsourcing.</t>
-        </is>
-      </c>
+          <t>One practical action for their main challenge that they can start this month.</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>next30</t>
+          <t>next90</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Next 30 days</t>
+          <t>Next 90 days</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -2560,48 +2582,14 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>One practical action for their main challenge that they can start this month.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>next90</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Next 90 days</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>280</v>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
           <t>A feasible step toward their 6–12 month goal.</t>
         </is>
       </c>
+      <c r="H11" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2613,7 +2601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2626,12 +2614,13 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="60" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>The text each answer contributes. Heading and 'Why this matters' are used by priority cards. For a Multi question, the MULTI row is used when more than one answer is selected. Mark Approved when reviewed.</t>
+          <t>The text each answer contributes. Heading and 'Why this matters' are used by priority cards. For a Multi question, the MULTI row is used when more than one answer is selected. Action names the central action of a priority card: when two priority cards share an Action, only the first is shown and the other's Merge note (Sections tab) is added to its reason. Mark Approved when reviewed.</t>
         </is>
       </c>
     </row>
@@ -2684,6 +2673,11 @@
       <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Reviewer notes</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>Action</t>
         </is>
       </c>
     </row>
@@ -2725,6 +2719,7 @@
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr"/>
+      <c r="K3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -2764,6 +2759,7 @@
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr"/>
+      <c r="K4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2803,6 +2799,7 @@
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2842,6 +2839,7 @@
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr"/>
+      <c r="K6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2881,6 +2879,7 @@
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr"/>
+      <c r="K7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2920,6 +2919,7 @@
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr"/>
+      <c r="K8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2959,6 +2959,7 @@
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr"/>
+      <c r="K9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2998,6 +2999,7 @@
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr"/>
+      <c r="K10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -3037,6 +3039,7 @@
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr"/>
+      <c r="K11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -3066,7 +3069,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Identify your most-used and highest-risk content and review it first for outdated information, accessibility gaps and parts you could reuse. Give each item a review date so upkeep becomes routine.</t>
+          <t>List your most-used and highest-risk content, and give each item an owner and a review date, so upkeep becomes routine rather than something done only when a problem is noticed.</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -3083,7 +3086,16 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>content-upkeep</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -3113,7 +3125,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Make demand visible in one backlog, agree how requests are prioritized, and build reusable templates and patterns so each new program takes less effort.</t>
+          <t>Make demand visible in one shared backlog and agree with stakeholders how requests are prioritized, so your team’s time goes to the work that matters most.</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -3130,7 +3142,16 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>intake-prioritization</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -3178,6 +3199,11 @@
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr"/>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>learner-application</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -3225,6 +3251,11 @@
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr"/>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>quality-governance</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -3272,6 +3303,11 @@
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>impact-measurement</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -3301,7 +3337,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Look at where time goes today, from request to launch, and remove the biggest bottlenecks before adding more programs. Reusable designs and clear sign-off steps add capacity without adding people.</t>
+          <t>Look at where time goes from request to launch and remove the biggest bottlenecks, such as unclear sign-off or repeated rework, before adding more programs.</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -3318,7 +3354,16 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>workflow-bottlenecks</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -3366,6 +3411,11 @@
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>reusable-production</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -3413,6 +3463,11 @@
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr"/>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>quality-governance</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -3460,6 +3515,11 @@
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>learner-application</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -3507,6 +3567,11 @@
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr"/>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>impact-measurement</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -3554,6 +3619,11 @@
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr"/>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>intake-prioritization</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -3583,7 +3653,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Pick the processes and templates that work best today and make them the default for new programs, with a short checklist for design and review.</t>
+          <t>Pick the planning and build steps that work best today and make them the default way every new program is run, so results depend less on who does the work.</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -3600,7 +3670,16 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr"/>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>standard-process</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -3648,6 +3727,11 @@
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr"/>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>portfolio-focus</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -3695,6 +3779,11 @@
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr"/>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>scale-evidence</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -3720,7 +3809,7 @@
       <c r="E26" s="5" t="inlineStr"/>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>You deliver learning through in-person sessions. Consider which parts could be supported with short reference materials or follow-up activities, so learning continues after the session.</t>
+          <t>You deliver learning through in-person sessions.</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr"/>
@@ -3733,7 +3822,12 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J26" s="5" t="inlineStr"/>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -3759,7 +3853,7 @@
       <c r="E27" s="5" t="inlineStr"/>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>You deliver learning through virtual live sessions. Keep sessions interactive and focused, and add simple follow-up materials so people can revisit key points.</t>
+          <t>You deliver learning through virtual live sessions.</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr"/>
@@ -3772,7 +3866,12 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J27" s="5" t="inlineStr"/>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -3798,7 +3897,7 @@
       <c r="E28" s="5" t="inlineStr"/>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>You use self-paced eLearning. Review your most-used modules regularly for outdated examples and accessibility gaps, and look for content you could reuse across courses.</t>
+          <t>You use self-paced eLearning.</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
@@ -3811,7 +3910,12 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J28" s="5" t="inlineStr"/>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -3837,7 +3941,7 @@
       <c r="E29" s="5" t="inlineStr"/>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>You use microlearning and performance support. Make sure each resource is easy to find at the moment of need, and link related resources so they support a bigger goal.</t>
+          <t>You use microlearning and performance support.</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
@@ -3850,7 +3954,12 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J29" s="5" t="inlineStr"/>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -3876,7 +3985,7 @@
       <c r="E30" s="5" t="inlineStr"/>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>You use documents and reference materials. Keep them current, easy to search and clearly owned, and consider which topics would benefit from practice or guided learning.</t>
+          <t>You use documents and reference materials.</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr"/>
@@ -3889,7 +3998,12 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -3915,7 +4029,7 @@
       <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>You use several delivery methods: {Q3}. Identify where they can work together to support the same outcome, rather than planning each one separately.</t>
+          <t>You use several delivery methods: {Q3}.</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr"/>
@@ -3928,7 +4042,12 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J31" s="5" t="inlineStr"/>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -3968,6 +4087,7 @@
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr"/>
+      <c r="K32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -4007,6 +4127,7 @@
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr"/>
+      <c r="K33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -4046,6 +4167,7 @@
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr"/>
+      <c r="K34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -4085,16 +4207,17 @@
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr"/>
+      <c r="K35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>sourcing</t>
+          <t>next30</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -4104,13 +4227,13 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Mainly in-house: Mainly in-house, by our own people.</t>
+          <t>Content upkeep: Keeping existing learning content accurate, relevant and up to date.</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr"/>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Because most work is done in-house, document key processes and decisions so knowledge isn't held by only a few people.</t>
+          <t>List your most-used learning assets and note when each was last reviewed. Pick the two most out of date and schedule their review.</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr"/>
@@ -4124,16 +4247,17 @@
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr"/>
+      <c r="K36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>sourcing</t>
+          <t>next30</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -4143,13 +4267,13 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Mixed: By a mix of our own people and external partners.</t>
+          <t>Delivery capacity: Producing and delivering learning fast enough to meet demand.</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr"/>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>With work shared between your own people and partners, agree briefs, review steps and quality standards that both sides use.</t>
+          <t>Put every open learning request into one list with a requester, a deadline and a business reason, and agree the top priorities with stakeholders.</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr"/>
@@ -4163,16 +4287,17 @@
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr"/>
+      <c r="K37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>sourcing</t>
+          <t>next30</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -4182,13 +4307,13 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Mainly partners: Mainly by external partners.</t>
+          <t>Learner engagement: Getting people to take part in learning and apply it at work.</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr"/>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>As partners deliver most of the work, keep ownership of priorities, quality standards and final sign-off inside your organization.</t>
+          <t>Ask a few recent participants and their managers what they have used at work since the program, and note what got in the way.</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
@@ -4202,6 +4327,7 @@
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr"/>
+      <c r="K38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -4216,18 +4342,18 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Content upkeep: Keeping existing learning content accurate, relevant and up to date.</t>
+          <t>Consistent quality: Keeping quality consistent across programs, teams or regions.</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr"/>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>List your most-used learning assets and note when each was last reviewed. Pick the two most out of date and schedule their review.</t>
+          <t>Draft a one-page quality checklist and test it on two recent programs, ideally built by different people or partners.</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr"/>
@@ -4241,6 +4367,7 @@
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr"/>
+      <c r="K39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -4255,18 +4382,18 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Delivery capacity: Producing and delivering learning fast enough to meet demand.</t>
+          <t>Demonstrating impact: Showing how learning contributes to business results.</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr"/>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Put every open learning request into one list with a requester, a deadline and a business reason, and agree the top priorities with stakeholders.</t>
+          <t>Pick one priority program and agree with its business owner which measure it should influence and where the data will come from.</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr"/>
@@ -4280,32 +4407,33 @@
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr"/>
+      <c r="K40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>next30</t>
+          <t>next90</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Learner engagement: Getting people to take part in learning and apply it at work.</t>
+          <t>Delivery capacity: Increase delivery capacity.</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr"/>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Ask a few recent participants and their managers what they have used at work since the program, and note what got in the way.</t>
+          <t>Map how a typical program moves from request to launch, remove the biggest bottleneck, and agree clear sign-off steps for your most common requests.</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr"/>
@@ -4318,33 +4446,38 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="J41" s="5" t="inlineStr"/>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-11 (follow-up polish)</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>next30</t>
+          <t>next90</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Consistent quality: Keeping quality consistent across programs, teams or regions.</t>
+          <t>Faster development: Reduce development and update time.</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr"/>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Draft a one-page quality checklist and test it on two recent programs, ideally built by different people or partners.</t>
+          <t>Build a shared library of templates and reusable components, and organize source files so any program can be updated quickly.</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
@@ -4358,32 +4491,33 @@
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr"/>
+      <c r="K42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>next30</t>
+          <t>next90</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Demonstrating impact: Showing how learning contributes to business results.</t>
+          <t>Quality and consistency: Improve learning quality and consistency.</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr"/>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Pick one priority program and agree with its business owner which measure it should influence and where the data will come from.</t>
+          <t>Roll out a quality checklist to everyone who builds or reviews learning, and review a sample of programs against it at the end of the quarter.</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr"/>
@@ -4397,6 +4531,7 @@
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr"/>
+      <c r="K43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -4411,18 +4546,18 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Delivery capacity: Increase delivery capacity.</t>
+          <t>Engagement and application: Improve learner engagement and application.</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr"/>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Map how a typical program moves from request to launch, remove the biggest bottleneck, and create reusable templates for your most common requests.</t>
+          <t>Redesign one program with practice activities and manager follow-up, then compare participation, feedback and application with the previous version.</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr"/>
@@ -4436,6 +4571,7 @@
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr"/>
+      <c r="K44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -4450,18 +4586,18 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Faster development: Reduce development and update time.</t>
+          <t>Business impact: Demonstrate business impact.</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr"/>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Build a shared library of templates and reusable components, and organize source files so any program can be updated quickly.</t>
+          <t>Share the results of one evaluated program with its business owner, agree what the evidence does and doesn't show, and decide which program to evaluate next.</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr"/>
@@ -4475,127 +4611,11 @@
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>next90</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Quality and consistency: Improve learning quality and consistency.</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr"/>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>Roll out a quality checklist to everyone who builds or reviews learning, and review a sample of programs against it at the end of the quarter.</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr"/>
-      <c r="H46" s="5">
-        <f>LEN(F46)</f>
-        <v/>
-      </c>
-      <c r="I46" s="5" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="J46" s="5" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>next90</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Engagement and application: Improve learner engagement and application.</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr"/>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>Redesign one program with practice activities and manager follow-up, then compare participation, feedback and application with the previous version.</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr"/>
-      <c r="H47" s="5">
-        <f>LEN(F47)</f>
-        <v/>
-      </c>
-      <c r="I47" s="5" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="J47" s="5" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>next90</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Business impact: Demonstrate business impact.</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr"/>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>Share the results of one evaluated program with its business owner, agree what the evidence does and doesn't show, and decide which program to evaluate next.</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr"/>
-      <c r="H48" s="5">
-        <f>LEN(F48)</f>
-        <v/>
-      </c>
-      <c r="I48" s="5" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="J48" s="5" t="inlineStr"/>
+      <c r="K45" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="I3:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4612,7 +4632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4630,7 +4650,7 @@
     <row r="1" ht="60" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Overrides for specific combinations. 'When' uses Q-code=answer pairs joined by AND (for a Multi question, Q3=C means C is among the selections). Modes: Replace, Add before, Add after, Remove (hides the section). Higher Priority wins when two Replace rules hit the same section.</t>
+          <t>Overrides for specific combinations. 'When' uses Q-code=answer pairs joined by AND (for a Multi question, Q3=C means C is among the selections). Modes: Replace, Add before, Add after, Remove (hides the section). When several rules of the same mode match a section, only the one with the highest Priority applies (ties: the higher row).</t>
         </is>
       </c>
     </row>
@@ -4694,22 +4714,26 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Q2=A AND Q6=B</t>
+          <t>Q4=A AND Q5=A</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>priority_goal</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Remove</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Without a dedicated L&amp;D team, learning is likely handled by people in other roles. Agree who decides priorities and signs off content, and share simple templates so no one starts from scratch.</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n">
         <v>10</v>
       </c>
@@ -4720,7 +4744,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Content upkeep and faster updates are the same priority; show it once.</t>
+          <t>No dedicated team + mainly in-house: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -4732,28 +4756,28 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Q2=A AND Q6=B</t>
+          <t>Q4=A AND Q5=B</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>priority_challenge</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Add after</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>This is also the goal you set for the next 6–12 months, so it is listed once.</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr"/>
+          <t>Without a dedicated L&amp;D team, name an internal owner who decides priorities and signs off content, and give partners clear briefs so internal and external work fits together.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
@@ -4762,7 +4786,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Explains why the goal priority is missing.</t>
+          <t>No dedicated team + mixed sourcing: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -4774,22 +4798,26 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Q2=B AND Q6=A</t>
+          <t>Q4=A AND Q5=C</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>priority_goal</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Remove</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Name an internal owner to prioritize requests, brief partners and approve quality. Use a simple shared tracker to keep delivery visible.</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n">
         <v>10</v>
       </c>
@@ -4800,7 +4828,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Delivery capacity challenge and goal are the same priority.</t>
+          <t>No dedicated team + mainly partners: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -4812,28 +4840,28 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Q2=B AND Q6=A</t>
+          <t>Q4=B AND Q5=A</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>priority_challenge</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Add after</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>This is also the goal you set for the next 6–12 months, so it is listed once.</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
+          <t>Protect limited capacity with a prioritized backlog, reusable templates and documented handoffs, so work doesn’t depend on one person.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
@@ -4842,7 +4870,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Explains why the goal priority is missing.</t>
+          <t>Small team + mainly in-house: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -4854,22 +4882,26 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Q2=C AND Q6=D</t>
+          <t>Q4=B AND Q5=B</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>priority_goal</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Remove</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>With a small team working alongside partners, keep one prioritized backlog and decide early which work partners take on, with clear briefs and one shared review step.</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="n">
         <v>10</v>
       </c>
@@ -4880,7 +4912,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Engagement challenge and goal are the same priority.</t>
+          <t>Small team + mixed sourcing: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -4892,28 +4924,28 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Q2=C AND Q6=D</t>
+          <t>Q4=B AND Q5=C</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>priority_challenge</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Add after</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>This is also the goal you set for the next 6–12 months, so it is listed once.</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr"/>
+          <t>With a small team and partners doing most of the work, focus your team on prioritizing requests, briefing partners and approving quality rather than on production.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
@@ -4922,7 +4954,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Explains why the goal priority is missing.</t>
+          <t>Small team + mainly partners: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -4934,22 +4966,26 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Q2=D AND Q6=C</t>
+          <t>Q4=C AND Q5=A</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>priority_goal</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Remove</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
-      <c r="G9" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>With a medium-sized team working in-house, agree shared standards and documented handoffs so work stays consistent as it moves between people.</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n">
         <v>10</v>
       </c>
@@ -4960,7 +4996,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Quality challenge and goal are the same priority.</t>
+          <t>Medium team + mainly in-house: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -4972,28 +5008,28 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Q2=D AND Q6=C</t>
+          <t>Q4=C AND Q5=B</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>priority_challenge</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Add after</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>This is also the goal you set for the next 6–12 months, so it is listed once.</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr"/>
+          <t>Agree clear briefs, review responsibilities and handoffs across your team and partners so work stays consistent.</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
@@ -5002,7 +5038,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Explains why the goal priority is missing.</t>
+          <t>Medium team + mixed sourcing: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -5014,22 +5050,26 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Q2=E AND Q6=E</t>
+          <t>Q4=C AND Q5=C</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>priority_goal</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Remove</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr"/>
-      <c r="F11" s="5" t="inlineStr"/>
-      <c r="G11" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>With partners delivering most of the work, use your team to set standards, brief partners and review what comes back, so quality stays consistent across suppliers.</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n"/>
       <c r="H11" s="5" t="n">
         <v>10</v>
       </c>
@@ -5040,7 +5080,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Impact challenge and goal are the same priority.</t>
+          <t>Medium team + mainly partners: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -5052,28 +5092,28 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Q2=E AND Q6=E</t>
+          <t>Q4=D AND Q5=A</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>priority_challenge</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Add after</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>This is also the goal you set for the next 6–12 months, so it is listed once.</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr"/>
+          <t>With a large in-house team, make roles and review ownership clear across groups and keep one view of work in progress, so effort isn’t duplicated.</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
@@ -5082,7 +5122,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Explains why the goal priority is missing.</t>
+          <t>Large team + mainly in-house: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -5094,28 +5134,28 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Q2=A AND Q3=C</t>
+          <t>Q4=D AND Q5=B</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>delivery</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Add after</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>As content upkeep is your main challenge, start with your highest-use eLearning: check for outdated examples, accessibility gaps and reusable content.</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr"/>
+          <t>With a large team working alongside partners, agree shared quality standards, assign review and sign-off owners, and maintain one view of work in progress.</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="n"/>
       <c r="H13" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
@@ -5124,7 +5164,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>eLearning user with content upkeep challenge.</t>
+          <t>Large team + mixed sourcing: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -5136,28 +5176,28 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Q2=A AND Q3=E</t>
+          <t>Q4=D AND Q5=C</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>delivery</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Add after</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr"/>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Give each reference document an owner and a review date, so upkeep doesn't depend on someone noticing a problem.</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr"/>
+          <t>With a large team and partners delivering most of the work, give each partner relationship a clear owner and apply the same standards and sign-off to all of them.</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
@@ -5166,7 +5206,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Reference materials with content upkeep challenge.</t>
+          <t>Large team + mainly partners: one paragraph covering team size and sourcing together.</t>
         </is>
       </c>
     </row>
@@ -5178,7 +5218,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Q2=C AND Q3=D</t>
+          <t>Q2=A</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -5191,15 +5231,15 @@
           <t>Add after</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr"/>
+      <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Link each microlearning resource to the task it supports, so people can apply it at work.</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr"/>
+          <t>Start with your highest-use materials in each format and check them for outdated information, accessibility gaps and parts you could reuse.</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n"/>
       <c r="H15" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
@@ -5208,7 +5248,7 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Microlearning with engagement challenge.</t>
+          <t>Content upkeep: delivery advice that serves the main challenge, whatever the method mix.</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5260,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Q2=B AND Q3=A</t>
+          <t>Q2=B</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -5233,15 +5273,15 @@
           <t>Add after</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>If live sessions take much of your team's time, consider which could be recorded or supported with self-paced material.</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr"/>
+          <t>Look for content you rebuild for each request and turn it into reusable assets, so new work takes less effort whatever the format.</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
@@ -5250,7 +5290,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Capacity pressure with in-person delivery.</t>
+          <t>Delivery capacity: delivery advice that serves the main challenge, whatever the method mix.</t>
         </is>
       </c>
     </row>
@@ -5262,26 +5302,26 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Q4=A AND Q5=A</t>
+          <t>Q2=C</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>sourcing</t>
+          <t>delivery</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Replace</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr"/>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>As learning is handled in-house without a dedicated team, it is likely spread across other roles. Agree a simple way to share templates and decisions between them.</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr"/>
+          <t>Plan practice, participation and follow-up so people apply what they learn, rather than counting attendance or completion alone.</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n"/>
       <c r="H17" s="5" t="n">
         <v>10</v>
       </c>
@@ -5292,7 +5332,7 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>No dedicated team but in-house delivery: other internal roles do the work.</t>
+          <t>Learner engagement: delivery advice that serves the main challenge, whatever the method mix.</t>
         </is>
       </c>
     </row>
@@ -5304,26 +5344,26 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Q4=A AND Q5=C</t>
+          <t>Q2=D</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>team</t>
+          <t>delivery</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Replace</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr"/>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>You don't have a dedicated internal L&amp;D team and partners deliver most of the work, so name an internal owner who sets priorities, briefs partners and signs off quality.</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr"/>
+          <t>Apply the same quality and accessibility criteria to every format you use, with a few checks specific to each one.</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="n"/>
       <c r="H18" s="5" t="n">
         <v>10</v>
       </c>
@@ -5334,7 +5374,7 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>No internal team, partner-led delivery.</t>
+          <t>Consistent quality: delivery advice that serves the main challenge, whatever the method mix.</t>
         </is>
       </c>
     </row>
@@ -5346,26 +5386,26 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Q4=D AND Q5=B</t>
+          <t>Q2=E</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>sourcing</t>
+          <t>delivery</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Replace</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr"/>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>With a large team working alongside partners, clarify review ownership and quality standards across internal teams and partners, and keep one shared view of work in progress.</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr"/>
+          <t>For one priority program, choose a measure of application or performance and agree a baseline with its business owner. Attendance and completion figures alone won’t show impact.</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="n"/>
       <c r="H19" s="5" t="n">
         <v>10</v>
       </c>
@@ -5376,7 +5416,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Large hybrid team.</t>
+          <t>Demonstrating impact: delivery advice that serves the main challenge, whatever the method mix.</t>
         </is>
       </c>
     </row>
@@ -5388,28 +5428,28 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Q1=D AND Q6=E</t>
+          <t>Q2=E AND Q3=C</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>priority_goal</t>
+          <t>delivery</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Replace</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr"/>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Connect an existing learning measure to a relevant operational outcome, and agree with business owners how to evaluate the change.</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr"/>
+          <t>For your eLearning, choose a meaningful application or performance measure, agree a baseline with the business owner, and connect module activity to what changes at work. Completions alone won’t prove impact.</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="n"/>
       <c r="H20" s="5" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
@@ -5418,7 +5458,7 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Optimizing teams already measure; build on it rather than start from scratch.</t>
+          <t>Impact + eLearning: measurement, not module upkeep.</t>
         </is>
       </c>
     </row>
@@ -5430,28 +5470,28 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Q1=A AND Q6=E</t>
+          <t>Q2=A AND Q3=C</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>next90</t>
+          <t>delivery</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Add before</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr"/>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Start with one simple, agreed measure rather than a full evaluation framework.</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr"/>
+          <t>Start with your highest-use eLearning modules: check them for obsolete examples, accessibility gaps and content you could reuse across courses.</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="n"/>
       <c r="H21" s="5" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
@@ -5460,7 +5500,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Foundational teams seeking impact.</t>
+          <t>Content upkeep + eLearning.</t>
         </is>
       </c>
     </row>
@@ -5472,35 +5512,413 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
+          <t>Q2=A AND Q3=E</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Keep reference documents in one place with a visible last-reviewed date, so people can trust what they find.</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Content upkeep + reference materials (eLearning wins if both are selected).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>R21</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Q2=C AND Q3=A</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>In live sessions, build in practice, discussion and feedback, and plan a follow-up activity so people apply what they learned rather than just attend.</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Engagement + in-person ILT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>R22</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Q2=C AND Q3=B</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>In live sessions, build in practice, discussion and feedback, and plan a follow-up activity so people apply what they learned rather than just attend.</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="n"/>
+      <c r="H24" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Engagement + virtual ILT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>R23</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Q2=C AND Q3=D</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Link each microlearning resource to the task it supports, so people can find it and apply it at the moment of need.</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Engagement + microlearning (live sessions win if both are selected).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>R24</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Q2=B AND Q3=A</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Identify session content you repeat often and turn it into reusable facilitation assets, reference materials or optional self-paced support, so live time goes where it adds most.</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="n"/>
+      <c r="H26" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Capacity + in-person ILT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>R25</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Q2=B AND Q3=B</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Identify session content you repeat often and turn it into reusable facilitation assets, reference materials or optional self-paced support, so live time goes where it adds most.</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Capacity + virtual ILT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>R26</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Q2=B AND Q6=B</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Add after</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Reuse approved source content and design patterns across your formats, and keep clear ownership and version control so updates are quick.</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Capacity challenge + faster development goal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>R27</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Q1=D AND Q6=E</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>priority_goal</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Replace</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Connect an existing learning measure to a relevant operational outcome, and agree with business owners how to evaluate the change.</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Optimizing teams already measure; build on it rather than start from scratch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>R28</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Q1=A AND Q6=E</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>next90</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Add before</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Start with one simple, agreed measure rather than a full evaluation framework.</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>Foundational teams seeking impact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>R29</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
           <t>Q1=A AND Q6=A</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>next90</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>Add after</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr"/>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>Keep the process simple: a shared request list and one template are enough to start.</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="5" t="n">
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="J22" s="5" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>Foundational teams seeking capacity.</t>
         </is>

</xml_diff>